<commit_message>
Updated control files for new climate script field
</commit_message>
<xml_diff>
--- a/W3_LSPC_Watershed/inputs/Project_Control_Gualala.xlsx
+++ b/W3_LSPC_Watershed/inputs/Project_Control_Gualala.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E8C6EE4-32C6-4D4D-9954-476112D26768}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B41E313F-026F-44BF-A037-7D9356467196}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="79">
   <si>
     <t>flag</t>
   </si>
@@ -273,6 +273,12 @@
   </si>
   <si>
     <t>../data/projects/Gualala</t>
+  </si>
+  <si>
+    <t>other</t>
+  </si>
+  <si>
+    <t>raw/gage/other</t>
   </si>
 </sst>
 </file>
@@ -686,7 +692,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7E96793-80A0-4E7D-B9B3-D183DF1A597C}">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" customWidth="1"/>
@@ -870,13 +876,13 @@
         <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="C11" t="s">
-        <v>14</v>
+        <v>77</v>
       </c>
       <c r="D11" t="s">
-        <v>30</v>
+        <v>78</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -890,10 +896,10 @@
         <v>29</v>
       </c>
       <c r="C12" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -907,10 +913,10 @@
         <v>29</v>
       </c>
       <c r="C13" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -921,13 +927,13 @@
         <v>20</v>
       </c>
       <c r="B14" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C14" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D14" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -941,10 +947,10 @@
         <v>33</v>
       </c>
       <c r="C15" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="D15" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -955,13 +961,13 @@
         <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C16" t="s">
         <v>35</v>
       </c>
       <c r="D16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -972,13 +978,13 @@
         <v>20</v>
       </c>
       <c r="B17" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="C17" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D17" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -992,12 +998,29 @@
         <v>38</v>
       </c>
       <c r="C18" t="s">
+        <v>39</v>
+      </c>
+      <c r="D18" t="s">
+        <v>40</v>
+      </c>
+      <c r="E18" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" t="s">
+        <v>38</v>
+      </c>
+      <c r="C19" t="s">
         <v>41</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D19" t="s">
         <v>42</v>
       </c>
-      <c r="E18" t="b">
+      <c r="E19" t="b">
         <v>0</v>
       </c>
     </row>
@@ -7130,42 +7153,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"Blank Document","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="84c16208-172a-4eaa-b33e-1408ce0b909e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="04ff8bd0-14ef-4472-a603-3a4b6f9fed19">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <LastModifiedBy xmlns="04ff8bd0-14ef-4472-a603-3a4b6f9fed19">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </LastModifiedBy>
-    <LastModifiedOn xmlns="04ff8bd0-14ef-4472-a603-3a4b6f9fed19" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100AD1B9453B0FD26428396C40DDB69C7F0" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="7ae69fa2ec7ba05b1cd5ad5facbfed2a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="04ff8bd0-14ef-4472-a603-3a4b6f9fed19" xmlns:ns3="84c16208-172a-4eaa-b33e-1408ce0b909e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="593a7e08a14a0b523a37a1b36e06b6ea" ns2:_="" ns3:_="">
     <xsd:import namespace="04ff8bd0-14ef-4472-a603-3a4b6f9fed19"/>
@@ -7398,38 +7385,43 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{43BD7F1F-596C-48D7-B49B-C059BD9AD9F3}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06124858-FF52-43B6-9F5F-14F707108C35}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="84c16208-172a-4eaa-b33e-1408ce0b909e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="04ff8bd0-14ef-4472-a603-3a4b6f9fed19">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <LastModifiedBy xmlns="04ff8bd0-14ef-4472-a603-3a4b6f9fed19">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </LastModifiedBy>
+    <LastModifiedOn xmlns="04ff8bd0-14ef-4472-a603-3a4b6f9fed19" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A7D180A-E261-4A2D-8CBC-AEEBF9B497B3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="84c16208-172a-4eaa-b33e-1408ce0b909e"/>
-    <ds:schemaRef ds:uri="04ff8bd0-14ef-4472-a603-3a4b6f9fed19"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
 </file>
 
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{41E32FE7-C838-46D6-8359-8A7BBC9B619E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"Blank Document","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
 </file>
 
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91099A35-A67A-49FB-8DC5-AD08F2B17B2B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7448,6 +7440,37 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{41E32FE7-C838-46D6-8359-8A7BBC9B619E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A7D180A-E261-4A2D-8CBC-AEEBF9B497B3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="84c16208-172a-4eaa-b33e-1408ce0b909e"/>
+    <ds:schemaRef ds:uri="04ff8bd0-14ef-4472-a603-3a4b6f9fed19"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06124858-FF52-43B6-9F5F-14F707108C35}">
+  <ds:schemaRefs/>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{43BD7F1F-596C-48D7-B49B-C059BD9AD9F3}">
+  <ds:schemaRefs/>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{0bb6ca0c-ccb3-428b-9d5f-a9c60cad6645}" enabled="1" method="Standard" siteId="{fe186a25-7d49-41e6-9941-05d2281d36c1}" contentBits="0" removed="0"/>

</xml_diff>